<commit_message>
fix validatin bug in delivery time
</commit_message>
<xml_diff>
--- a/Phase_2_Operational_Data_Preparation_Excel/پروژه.xlsx
+++ b/Phase_2_Operational_Data_Preparation_Excel/پروژه.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EMTOO\Desktop\dars\ایتی\IT project\Phase_2_Operational_Data_Preparation_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1560DE88-5711-4256-B94D-14525DB85A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FA1660-747B-45D4-978B-B421EB27F9EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product_Table" sheetId="2" r:id="rId1"/>
@@ -593,20 +593,12 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="8"/>
-      <c r="E2" s="10">
-        <v>46368</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="E3" s="10">
-        <v>46003</v>
-      </c>
     </row>
     <row r="8" spans="1:9">
       <c r="D8" s="6"/>
     </row>
   </sheetData>
-  <dataValidations count="10">
+  <dataValidations count="11">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="بیبلیلیلیلی" sqref="B1" xr:uid="{C7CF2BF0-4B8B-4A5C-BADB-A3E1FEE1FECF}"/>
     <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Product Name" error="Only letters are allowed; no numbers or symbols." promptTitle="Product Name" prompt="Enter the name (Letters only)." sqref="B2:B1048576" xr:uid="{C816AF5D-481B-4A00-B8D4-FC675BEB1935}">
       <formula1>AND(B2&lt;&gt;"",SUMPRODUCT(--ISNUMBER(FIND(MID(B2,ROW(INDIRECT("1:"&amp;LEN(B2))),1),"ABCDEFGHIJKLMNOPQRSTUVWXYZabcdefghijklmnopqrstuvwxyz ")))=LEN(B2))</formula1>
@@ -625,7 +617,7 @@
       <formula1>45658</formula1>
       <formula2>47847</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1:F1048576" xr:uid="{BA4DFE87-23BC-4D6D-A893-3D701ED8DFD0}">
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1" xr:uid="{BA4DFE87-23BC-4D6D-A893-3D701ED8DFD0}">
       <formula1>E2</formula1>
     </dataValidation>
     <dataValidation type="whole" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Unit Quantity" error="Please enter a whole number between 1 and 100._x000a_" promptTitle="Unit Quantity" prompt="Enter a whole number between 1 and 100._x000a_" sqref="G1:G1048576" xr:uid="{03E8A2E4-1B5C-4F62-B3DC-D8EA8BAE5906}">
@@ -637,6 +629,9 @@
     </dataValidation>
     <dataValidation type="custom" operator="greaterThan" showInputMessage="1" showErrorMessage="1" errorTitle=" Invalid Unit Price" error="Unit Price must be a positive number with a maximum of 2 decimal places._x000a_" promptTitle="Unit Price" prompt="Unit Price must be a positive number with a maximum of 2 decimal places._x000a_" sqref="H2:H1048576" xr:uid="{459525FE-0763-4A7B-80EE-24DDBD9384DE}">
       <formula1>AND(ISNUMBER(H2),H2&gt;0,ROUND(H2,2)=H2)</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{2552F9F0-9916-420F-8D92-02D084C9CFDD}">
+      <formula1>E2</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>